<commit_message>
Add points for 6zhd6pt8kyzrbkgwq2i2k8u1g_playerlog
</commit_message>
<xml_diff>
--- a/bnc-streamlit-app/data/points/6zhd6pt8kyzrbkgwq2i2k8u1g_playerlog.xlsx
+++ b/bnc-streamlit-app/data/points/6zhd6pt8kyzrbkgwq2i2k8u1g_playerlog.xlsx
@@ -780,14 +780,14 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="n">
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
@@ -816,7 +816,7 @@
         </is>
       </c>
       <c r="AD2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE2" t="n">
         <v>0</v>
@@ -835,7 +835,7 @@
         <v>0</v>
       </c>
       <c r="AM2" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="AN2" t="n">
         <v>0</v>
@@ -850,7 +850,7 @@
         <v>0</v>
       </c>
       <c r="AR2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS2" t="n">
         <v>0</v>
@@ -955,14 +955,14 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="n">
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
@@ -991,7 +991,7 @@
         </is>
       </c>
       <c r="AD3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE3" t="n">
         <v>0</v>
@@ -1008,21 +1008,21 @@
         </is>
       </c>
       <c r="AI3" t="n">
-        <v>-0.1587343</v>
+        <v>-0.11569904</v>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>-0.29</t>
+          <t>-0.31</t>
         </is>
       </c>
       <c r="AK3" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="AL3" t="n">
         <v>0</v>
       </c>
       <c r="AM3" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="AN3" t="n">
         <v>0</v>
@@ -1142,14 +1142,14 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="n">
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="S4" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
@@ -1178,7 +1178,7 @@
         </is>
       </c>
       <c r="AD4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE4" t="n">
         <v>0</v>
@@ -1195,30 +1195,30 @@
         </is>
       </c>
       <c r="AI4" t="n">
-        <v>0.12968152</v>
+        <v>0.94467989</v>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>-0.01</t>
+          <t>+0.75</t>
         </is>
       </c>
       <c r="AK4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="AL4" t="n">
         <v>0</v>
       </c>
       <c r="AM4" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="AN4" t="n">
         <v>0</v>
       </c>
       <c r="AO4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ4" t="n">
         <v>0</v>
@@ -1227,7 +1227,7 @@
         <v>0</v>
       </c>
       <c r="AS4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT4" t="n">
         <v>1</v>
@@ -1264,7 +1264,7 @@
         <v>0</v>
       </c>
       <c r="BF4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG4" t="n">
         <v>0</v>
@@ -1325,14 +1325,14 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="n">
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
@@ -1340,7 +1340,7 @@
         </is>
       </c>
       <c r="S5" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
@@ -1361,7 +1361,7 @@
         </is>
       </c>
       <c r="AD5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE5" t="n">
         <v>0</v>
@@ -1378,21 +1378,21 @@
         </is>
       </c>
       <c r="AI5" t="n">
-        <v>0.22725346</v>
+        <v>0.30097492</v>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>+0.09</t>
+          <t>+0.11</t>
         </is>
       </c>
       <c r="AK5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AL5" t="n">
         <v>0</v>
       </c>
       <c r="AM5" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="AN5" t="n">
         <v>0</v>
@@ -1407,7 +1407,7 @@
         <v>0</v>
       </c>
       <c r="AR5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS5" t="n">
         <v>1</v>
@@ -1448,7 +1448,7 @@
         </is>
       </c>
       <c r="BE5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BF5" t="n">
         <v>0</v>
@@ -1512,14 +1512,14 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="n">
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -1527,7 +1527,7 @@
         </is>
       </c>
       <c r="S6" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
@@ -1548,7 +1548,7 @@
         </is>
       </c>
       <c r="AD6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE6" t="n">
         <v>0</v>
@@ -1565,11 +1565,11 @@
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>0.28876565</v>
+        <v>0.63536079</v>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>+0.15</t>
+          <t>+0.44</t>
         </is>
       </c>
       <c r="AK6" t="n">
@@ -1579,7 +1579,7 @@
         <v>0</v>
       </c>
       <c r="AM6" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="AN6" t="n">
         <v>0</v>
@@ -1597,10 +1597,10 @@
         <v>2</v>
       </c>
       <c r="AS6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU6" t="n">
         <v>1</v>
@@ -1635,7 +1635,7 @@
         </is>
       </c>
       <c r="BE6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BF6" t="n">
         <v>0</v>
@@ -1699,14 +1699,14 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="n">
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
@@ -1714,7 +1714,7 @@
         </is>
       </c>
       <c r="S7" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
@@ -1735,7 +1735,7 @@
         </is>
       </c>
       <c r="AD7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE7" t="n">
         <v>0</v>
@@ -1752,21 +1752,21 @@
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>0.14985989</v>
+        <v>0.26103138</v>
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>+0.01</t>
+          <t>+0.07</t>
         </is>
       </c>
       <c r="AK7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AL7" t="n">
         <v>0</v>
       </c>
       <c r="AM7" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="AN7" t="n">
         <v>0</v>
@@ -1781,10 +1781,10 @@
         <v>0</v>
       </c>
       <c r="AR7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AT7" t="n">
         <v>0</v>
@@ -1822,7 +1822,7 @@
         </is>
       </c>
       <c r="BE7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BF7" t="n">
         <v>0</v>
@@ -1886,14 +1886,14 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="n">
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -1901,7 +1901,7 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
@@ -1922,7 +1922,7 @@
         </is>
       </c>
       <c r="AD8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE8" t="n">
         <v>0</v>
@@ -1939,21 +1939,21 @@
         </is>
       </c>
       <c r="AI8" t="n">
-        <v>0.03867826000000001</v>
+        <v>0.13105376</v>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>-0.10</t>
+          <t>-0.06</t>
         </is>
       </c>
       <c r="AK8" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="AL8" t="n">
         <v>0</v>
       </c>
       <c r="AM8" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="AN8" t="n">
         <v>0</v>
@@ -1968,7 +1968,7 @@
         <v>0</v>
       </c>
       <c r="AR8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AS8" t="n">
         <v>1</v>
@@ -2069,14 +2069,14 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="n">
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
@@ -2084,7 +2084,7 @@
         </is>
       </c>
       <c r="S9" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
@@ -2105,7 +2105,7 @@
         </is>
       </c>
       <c r="AD9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE9" t="n">
         <v>0</v>
@@ -2122,21 +2122,21 @@
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>0.15360126</v>
+        <v>0.25693374</v>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>+0.02</t>
+          <t>+0.06</t>
         </is>
       </c>
       <c r="AK9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AL9" t="n">
         <v>0</v>
       </c>
       <c r="AM9" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="AN9" t="n">
         <v>0</v>
@@ -2256,14 +2256,14 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="n">
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -2271,7 +2271,7 @@
         </is>
       </c>
       <c r="S10" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
@@ -2292,7 +2292,7 @@
         </is>
       </c>
       <c r="AD10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE10" t="n">
         <v>0</v>
@@ -2309,21 +2309,21 @@
         </is>
       </c>
       <c r="AI10" t="n">
-        <v>0.8739235299999999</v>
+        <v>0.6680151</v>
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>+0.74</t>
+          <t>+0.47</t>
         </is>
       </c>
       <c r="AK10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AL10" t="n">
         <v>0</v>
       </c>
       <c r="AM10" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="AN10" t="n">
         <v>0</v>
@@ -2443,14 +2443,14 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="n">
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -2458,7 +2458,7 @@
         </is>
       </c>
       <c r="S11" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
@@ -2479,7 +2479,7 @@
         </is>
       </c>
       <c r="AD11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE11" t="n">
         <v>0</v>
@@ -2496,24 +2496,24 @@
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>0.2232297</v>
+        <v>1.11324512</v>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>+0.09</t>
+          <t>+0.92</t>
         </is>
       </c>
       <c r="AK11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AL11" t="n">
         <v>0</v>
       </c>
       <c r="AM11" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="AN11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO11" t="n">
         <v>0</v>
@@ -2525,7 +2525,7 @@
         <v>2</v>
       </c>
       <c r="AR11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS11" t="n">
         <v>0</v>
@@ -2540,7 +2540,7 @@
         <v>0</v>
       </c>
       <c r="AW11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX11" t="n">
         <v>0</v>
@@ -2555,7 +2555,7 @@
         <v>0</v>
       </c>
       <c r="BB11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BC11" t="n">
         <v>0</v>
@@ -2566,13 +2566,13 @@
         </is>
       </c>
       <c r="BE11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BF11" t="n">
+        <v>3</v>
+      </c>
+      <c r="BG11" t="n">
         <v>2</v>
-      </c>
-      <c r="BG11" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -2630,14 +2630,14 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="n">
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -2645,7 +2645,7 @@
         </is>
       </c>
       <c r="S12" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
@@ -2666,7 +2666,7 @@
         </is>
       </c>
       <c r="AD12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE12" t="n">
         <v>0</v>
@@ -2683,21 +2683,21 @@
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>0.10882551</v>
+        <v>0.36856311</v>
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>-0.03</t>
+          <t>+0.17</t>
         </is>
       </c>
       <c r="AK12" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="AL12" t="n">
         <v>0</v>
       </c>
       <c r="AM12" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="AN12" t="n">
         <v>0</v>
@@ -2712,7 +2712,7 @@
         <v>0</v>
       </c>
       <c r="AR12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS12" t="n">
         <v>0</v>
@@ -2721,7 +2721,7 @@
         <v>0</v>
       </c>
       <c r="AU12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AV12" t="n">
         <v>0</v>
@@ -2813,14 +2813,14 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="n">
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
@@ -2828,7 +2828,7 @@
         </is>
       </c>
       <c r="S13" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
@@ -2852,7 +2852,7 @@
         <v>0</v>
       </c>
       <c r="AE13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF13" t="n">
         <v>0</v>
@@ -2868,7 +2868,7 @@
         <v>0</v>
       </c>
       <c r="AM13" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="AN13" t="n">
         <v>0</v>
@@ -2984,14 +2984,14 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="n">
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
@@ -2999,7 +2999,7 @@
         </is>
       </c>
       <c r="S14" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
@@ -3023,10 +3023,10 @@
         <v>0</v>
       </c>
       <c r="AE14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF14" t="n">
-        <v>-0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG14" t="n">
         <v>1</v>
@@ -3037,21 +3037,21 @@
         </is>
       </c>
       <c r="AI14" t="n">
-        <v>0.3808046199999999</v>
+        <v>-0.1066331500000001</v>
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
-          <t>+0.25</t>
+          <t>-0.30</t>
         </is>
       </c>
       <c r="AK14" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="AL14" t="n">
         <v>0</v>
       </c>
       <c r="AM14" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="AN14" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
         <v>0</v>
       </c>
       <c r="AX14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY14" t="n">
         <v>0</v>
@@ -3167,14 +3167,14 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="n">
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
@@ -3182,7 +3182,7 @@
         </is>
       </c>
       <c r="S15" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
@@ -3206,10 +3206,10 @@
         <v>0</v>
       </c>
       <c r="AE15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF15" t="n">
-        <v>-0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG15" t="n">
         <v>1</v>
@@ -3220,21 +3220,21 @@
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>0.12972356</v>
+        <v>-0.04713017000000002</v>
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t>-0.01</t>
+          <t>-0.24</t>
         </is>
       </c>
       <c r="AK15" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="AL15" t="n">
         <v>0</v>
       </c>
       <c r="AM15" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="AN15" t="n">
         <v>0</v>
@@ -3350,14 +3350,14 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="n">
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="S16" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
@@ -3389,10 +3389,10 @@
         <v>0</v>
       </c>
       <c r="AE16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF16" t="n">
-        <v>-0</v>
+        <v>-0.05</v>
       </c>
       <c r="AG16" t="n">
         <v>1</v>
@@ -3403,21 +3403,21 @@
         </is>
       </c>
       <c r="AI16" t="n">
-        <v>0.04112503000000002</v>
+        <v>-0.14525429</v>
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
-          <t>-0.09</t>
+          <t>-0.34</t>
         </is>
       </c>
       <c r="AK16" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="AL16" t="n">
         <v>0</v>
       </c>
       <c r="AM16" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="AN16" t="n">
         <v>0</v>
@@ -3533,14 +3533,14 @@
         </is>
       </c>
       <c r="N17" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="n">
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
         </is>
       </c>
       <c r="S17" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
@@ -3572,10 +3572,10 @@
         <v>0</v>
       </c>
       <c r="AE17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF17" t="n">
-        <v>-0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG17" t="n">
         <v>1</v>
@@ -3586,21 +3586,21 @@
         </is>
       </c>
       <c r="AI17" t="n">
-        <v>0.07933372999999999</v>
+        <v>-0.08749384000000002</v>
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>-0.06</t>
+          <t>-0.28</t>
         </is>
       </c>
       <c r="AK17" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="AL17" t="n">
         <v>0</v>
       </c>
       <c r="AM17" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="AN17" t="n">
         <v>0</v>
@@ -3716,14 +3716,14 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="n">
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
@@ -3731,7 +3731,7 @@
         </is>
       </c>
       <c r="S18" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
@@ -3755,10 +3755,10 @@
         <v>0</v>
       </c>
       <c r="AE18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF18" t="n">
-        <v>-0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG18" t="n">
         <v>1</v>
@@ -3769,21 +3769,21 @@
         </is>
       </c>
       <c r="AI18" t="n">
-        <v>0.41495335</v>
+        <v>0.2354502</v>
       </c>
       <c r="AJ18" t="inlineStr">
         <is>
-          <t>+0.28</t>
+          <t>+0.04</t>
         </is>
       </c>
       <c r="AK18" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="AL18" t="n">
         <v>0</v>
       </c>
       <c r="AM18" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="AN18" t="n">
         <v>0</v>
@@ -3810,7 +3810,7 @@
         <v>1</v>
       </c>
       <c r="AV18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW18" t="n">
         <v>0</v>
@@ -3899,14 +3899,14 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="n">
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
@@ -3914,7 +3914,7 @@
         </is>
       </c>
       <c r="S19" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
@@ -3938,7 +3938,7 @@
         <v>0</v>
       </c>
       <c r="AE19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF19" t="n">
         <v>0</v>
@@ -3952,21 +3952,21 @@
         </is>
       </c>
       <c r="AI19" t="n">
-        <v>0.0143409</v>
+        <v>0.0240099</v>
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
-          <t>-0.12</t>
+          <t>-0.17</t>
         </is>
       </c>
       <c r="AK19" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="AL19" t="n">
         <v>0</v>
       </c>
       <c r="AM19" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="AN19" t="n">
         <v>0</v>
@@ -3993,7 +3993,7 @@
         <v>0</v>
       </c>
       <c r="AV19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AW19" t="n">
         <v>0</v>
@@ -4082,14 +4082,14 @@
         </is>
       </c>
       <c r="N20" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="n">
         <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
@@ -4097,7 +4097,7 @@
         </is>
       </c>
       <c r="S20" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
@@ -4121,10 +4121,10 @@
         <v>0</v>
       </c>
       <c r="AE20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF20" t="n">
-        <v>-0</v>
+        <v>-0.05</v>
       </c>
       <c r="AG20" t="n">
         <v>1</v>
@@ -4135,21 +4135,21 @@
         </is>
       </c>
       <c r="AI20" t="n">
-        <v>0.02778284000000002</v>
+        <v>0.06570752000000001</v>
       </c>
       <c r="AJ20" t="inlineStr">
         <is>
-          <t>-0.11</t>
+          <t>-0.13</t>
         </is>
       </c>
       <c r="AK20" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="AL20" t="n">
         <v>0</v>
       </c>
       <c r="AM20" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="AN20" t="n">
         <v>0</v>
@@ -4164,7 +4164,7 @@
         <v>0</v>
       </c>
       <c r="AR20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AS20" t="n">
         <v>1</v>
@@ -4265,14 +4265,14 @@
         </is>
       </c>
       <c r="N21" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="n">
         <v>0</v>
       </c>
       <c r="Q21" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
@@ -4280,7 +4280,7 @@
         </is>
       </c>
       <c r="S21" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
@@ -4304,7 +4304,7 @@
         <v>0</v>
       </c>
       <c r="AE21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF21" t="n">
         <v>0</v>
@@ -4318,21 +4318,21 @@
         </is>
       </c>
       <c r="AI21" t="n">
-        <v>-0.03267428000000001</v>
+        <v>-0.008937310000000018</v>
       </c>
       <c r="AJ21" t="inlineStr">
         <is>
-          <t>-0.17</t>
+          <t>-0.20</t>
         </is>
       </c>
       <c r="AK21" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="AL21" t="n">
         <v>0</v>
       </c>
       <c r="AM21" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="AN21" t="n">
         <v>0</v>
@@ -4448,14 +4448,14 @@
         </is>
       </c>
       <c r="N22" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="n">
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
@@ -4463,7 +4463,7 @@
         </is>
       </c>
       <c r="S22" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr"/>
@@ -4487,10 +4487,10 @@
         <v>0</v>
       </c>
       <c r="AE22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF22" t="n">
-        <v>-0</v>
+        <v>-0.05</v>
       </c>
       <c r="AG22" t="n">
         <v>1</v>
@@ -4501,21 +4501,21 @@
         </is>
       </c>
       <c r="AI22" t="n">
-        <v>0.0868236</v>
+        <v>0.02256683999999998</v>
       </c>
       <c r="AJ22" t="inlineStr">
         <is>
-          <t>-0.05</t>
+          <t>-0.17</t>
         </is>
       </c>
       <c r="AK22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AL22" t="n">
         <v>0</v>
       </c>
       <c r="AM22" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -4631,14 +4631,14 @@
         </is>
       </c>
       <c r="N23" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="n">
         <v>0</v>
       </c>
       <c r="Q23" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R23" t="inlineStr">
         <is>
@@ -4646,7 +4646,7 @@
         </is>
       </c>
       <c r="S23" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
@@ -4670,7 +4670,7 @@
         <v>0</v>
       </c>
       <c r="AE23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF23" t="n">
         <v>0</v>
@@ -4684,21 +4684,21 @@
         </is>
       </c>
       <c r="AI23" t="n">
-        <v>-0.02712260000000002</v>
+        <v>-0.02745209000000001</v>
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
-          <t>-0.16</t>
+          <t>-0.22</t>
         </is>
       </c>
       <c r="AK23" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="AL23" t="n">
         <v>0</v>
       </c>
       <c r="AM23" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="AN23" t="n">
         <v>0</v>
@@ -4713,7 +4713,7 @@
         <v>3</v>
       </c>
       <c r="AR23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS23" t="n">
         <v>0</v>

</xml_diff>